<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-03 Le pain chaud de Victorino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-03.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>cuisine au pain du village, classe, puis nappe du soir</t>
+          <t>école puis maison, sac de pain, nappe à carreaux, four du village, vélo au loin</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, papa, maman, maîtresse</t>
+          <t>Victorino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut découper un rond de papier comme le pain tiède. À l'école il écoute et pose les ciseaux. Un chuchotement serre son ventre. Le soir, il raconte, et les deux ronds se regardent sur la nappe.</t>
+          <t>Une odeur de croûte traverse la rue. Sur le pain du four, un éclat de croûte brille. Victorino veut raconter le vélo maintenant. Il coupe papa : les mots se perdent. À l'école, un camarade parle près de l'oreille : le ventre se noue, tout dire d'un coup échoue. Il refuse de foncer, attend, raconte près du pain. Merci vécu. Sur la croûte, l'éclat de croûte garde une trace.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le sac de pain craque encore un peu. Une miette tombe sur la nappe à carreaux. Ça sent le four du village. La rue est calme, tout près. Un vélo passe au loin, tout léger. Papa coupe une tartine. La croûte est dorée. Maman verse un peu de lait. Le pain est encore tiède, tu sens ? Une petite miette a voyagé jusqu'à la nappe. En ce moment, Victorino touche la croûte tiède. Elle est chaude, papa. Une bouchée, puis on part. Victorino croque. La croûte fait un petit bruit. À l'école, je veux découper un rond. Un rond comme le pain. Tu essuies tes doigts d'abord. Victorino passe le torchon. Le lait laisse une petite moustache blanche. Viens. J'essuie. Merci, maman. Le village sent le pain, ce matin. Tu as entendu le vélo, tout à l'heure ? Oui. Il était loin. Tu dis bonjour à la maîtresse. Oui. L'école sent le papier et le savon des mains. Les chaises font un petit bruit sur le sol. Bonjour. On range les ciseaux, maintenant. Bonjour, maîtresse. Victorino écoute. Il pose les ciseaux dans le pot, les pointes en bas. Merci. Maintenant, on découpe un rond. Victorino prend une feuille. Il suit la ligne, tout doux. Le rond tombe sur la table. Il ressemble au pain. Oui, Victorino. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près de l'oreille. Victorino sent un malaise. Son ventre se serre, comme un nœud. Il reste assis. Il pose le rond de papier près du pot. Les ciseaux brillent dans le pot, tout sages. Le soir, le sac de pain est encore sur la table. Ça sent le cacao et la croûte. La porte s'ouvre. Te voilà. Tu as faim ? Victorino pose le rond de papier sur la nappe. À côté de la miette. Le ventre est encore serré.</t>
+          <t>Une odeur de croûte traverse la rue. Le four du village respire, chaud. Un vélo passe au loin. Ding. Victorino connaît cette table. La nappe à carreaux est rouge et blanche. Sur la table, le sac de pain craque. Le papier du sac est chaud, un peu rêche. Papa coupe une tartine. La croûte est dorée, un peu cassante. Sur la croûte, un éclat de croûte brille. Il est doré, papa. C'est le four, Victorino. Tu sens le pain, toi ? Oui, maman. Je veux le dire, maintenant ! Papa parle à maman, près du lait. Le vélo a sonné, dans la rue. Oui, il était loin. Papa, le vélo ! Les mots de Victorino se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose ? Le vélo, il a sonné ! Victorino parle trop vite. Les mots tombent, mélangés. Oh. Le sourire de Victorino disparaît. L'éclat de croûte tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le pain ? En ce moment, Victorino serre le sac. Le papier reste chaud sous les doigts. Tu essuies tes doigts ? Oui. Maman verse un peu de lait. Une moustache blanche reste sur la lèvre. Une miette dore un carreau rouge. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, la rue sent le four. Le vélo n'est plus là. L'école sent le papier et le savon. Les chaises font un petit bruit. Victorino s'assoit près du pot. Les ciseaux brillent, pointes en bas. Il veut raconter le vélo. Le vélo a sonné, dans la rue ! Sa voix se cogne à la classe. Personne ne comprend le vélo. Victorino referme la bouche. Un camarade s'approche. Il parle près de l'oreille. Victorino sent un malaise. Son ventre se serre, comme un nœud. Je veux le dire, maintenant. Il ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Victorino reste assis. Le nœud reste dans le ventre. Le soir, le sac de pain est sur la table. Ça sent le cacao et la croûte. La nappe à carreaux attend. La porte s'ouvre. Te voilà. Tu as faim ? Victorino pose le cartable. Le ventre est serré, tout petit. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le sac de pain craque encore un peu. Une miette tombe sur la nappe à carreaux. Ça sent le four du village. La rue est calme, tout près. Un vélo passe au loin, tout léger. Papa coupe une tartine. La croûte est dorée. Maman verse un peu de lait. Le pain est encore tiède, tu sens ? Une petite miette a voyagé jusqu'à la nappe. En ce moment, Victorino touche la croûte tiède. Elle est chaude, papa. Une bouchée, puis on part. Victorino croque. La croûte fait un petit bruit. À l'école, je veux découper un rond. Un rond comme le pain. Tu essuies tes doigts d'abord. Victorino passe le torchon. Le lait laisse une petite moustache blanche. Viens. J'essuie. Merci, maman. Le village sent le pain, ce matin. Tu as entendu le vélo, tout à l'heure ? Oui. Il était loin. Tu dis bonjour à la maîtresse. Oui. L'école sent le papier et le savon des mains. Les chaises font un petit bruit sur le sol. Bonjour. On range les ciseaux, maintenant. Bonjour, maîtresse. Victorino écoute. Il pose les ciseaux dans le pot, les pointes en bas. Merci. Maintenant, on découpe un rond. Victorino prend une feuille. Il suit la ligne, tout doux. Le rond tombe sur la table. Il ressemble au pain. Oui, Victorino. Plus tard, quelqu'un s'approche. Une voix parle tout bas, tout près de l'oreille. Victorino sent un malaise. Son ventre se serre, comme un nœud. Il reste assis. Il pose le rond de papier près du pot. Les ciseaux brillent dans le pot, tout sages. Le soir, le sac de pain est encore sur la table. Ça sent le cacao et la croûte. La porte s'ouvre. Te voilà. Tu as faim ? Victorino pose le rond de papier sur la nappe. À côté de la miette. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une odeur de croûte traverse la rue. Le four du village respire, chaud. Un vélo passe au loin. Ding. Victorino connaît cette table. La nappe à carreaux est rouge et blanche. Sur la table, le sac de pain craque. Le papier du sac est chaud, un peu rêche. Papa coupe une tartine. La croûte est dorée, un peu cassante. Sur la croûte, un &lt;emphasis level="moderate"&gt;éclat de croûte&lt;/emphasis&gt; brille. Il est doré, papa. C'est le four, Victorino. Tu sens le pain, toi ? Oui, maman. Je veux le dire, maintenant ! Papa parle à maman, près du lait. Le vélo a sonné, dans la rue. Oui, il était loin. Papa, le vélo ! Les mots de Victorino se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose ? Le vélo, il a sonné ! Victorino parle trop vite. Les mots tombent, mélangés. Oh. Le sourire de Victorino disparaît. L'éclat de croûte tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le pain ? En ce moment, Victorino serre le sac. Le papier reste chaud sous les doigts. Tu essuies tes doigts ? Oui. Maman verse un peu de lait. Une moustache blanche reste sur la lèvre. Une miette dore un carreau rouge. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, la rue sent le four. Le vélo n'est plus là. L'école sent le papier et le savon. Les chaises font un petit bruit. Victorino s'assoit près du pot. Les ciseaux brillent, pointes en bas. Il veut raconter le vélo. Le vélo a sonné, dans la rue ! Sa voix se cogne à la classe. Personne ne comprend le vélo. Victorino referme la bouche. Un camarade s'approche. Il parle près de l'oreille. Victorino sent un malaise. Son ventre se serre, comme un nœud. Je veux le dire, maintenant. Il ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Victorino reste assis. Le nœud reste dans le ventre. Le soir, le sac de pain est sur la table. Ça sent le cacao et la croûte. La nappe à carreaux attend. La porte s'ouvre. Te voilà. Tu as faim ? Victorino pose le cartable. Le ventre est serré, tout petit. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nino est à l'école. La maîtresse parle. Nino aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les ciseaux. Nino range. Il écoute bien. Plus tard, un camarade chuchote. Il dit : garde ça. Nino sent un malaise. Son ventre est serré. Le soir, maman l'attend. Nino vient raconter à la maison. Il dit : j'ai eu un malaise. Maman écoute. Maman dit : tu as bien fait. On aime écouter. Si tu as un malaise, tu viens raconter à la maison. [pause]</t>
+          <t>Une odeur de croûte traverse la rue. Le four du village respire, chaud. Un vélo passe au loin. Ding. Victorino connaît cette table. La nappe à carreaux est rouge et blanche. Sur la table, le sac de pain craque. Le papier du sac est chaud, un peu rêche. Papa coupe une tartine. La croûte est dorée, un peu cassante. Sur la croûte, un &lt;emphasis&gt;éclat de croûte&lt;/emphasis&gt; brille. Il est doré, papa. C'est le four, Victorino. Tu sens le pain, toi ? Oui, maman. Je veux le dire, maintenant ! Papa parle à maman, près du lait. Le vélo a sonné, dans la rue. Oui, il était loin. Papa, le vélo ! Les mots de Victorino se cognent aux leurs. Personne ne tourne la tête. Tu disais quelque chose ? Le vélo, il a sonné ! Victorino parle trop vite. Les mots tombent, mélangés. Oh. Le sourire de Victorino disparaît. L'éclat de croûte tremble, puis tient. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes le pain ? En ce moment, Victorino serre le sac. Le papier reste chaud sous les doigts. Tu essuies tes doigts ? Oui. Maman verse un peu de lait. Une moustache blanche reste sur la lèvre. Une miette dore un carreau rouge. On y va ? On y va. Au revoir, maman. Au revoir, Victorino. Dehors, la rue sent le four. Le vélo n'est plus là. L'école sent le papier et le savon. Les chaises font un petit bruit. Victorino s'assoit près du pot. Les ciseaux brillent, pointes en bas. Il veut raconter le vélo. Le vélo a sonné, dans la rue ! Sa voix se cogne à la classe. Personne ne comprend le vélo. Victorino referme la bouche. Un camarade s'approche. Il parle près de l'oreille. Victorino sent un malaise. Son ventre se serre, comme un nœud. Je veux le dire, maintenant. Il ouvre la bouche, trop vite. Les mots se perdent dans la classe. Personne n'entend le malaise. Victorino reste assis. Le nœud reste dans le ventre. Le soir, le sac de pain est sur la table. Ça sent le cacao et la croûte. La nappe à carreaux attend. La porte s'ouvre. Te voilà. Tu as faim ? Victorino pose le cartable. Le ventre est serré, tout petit. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de croûte</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,72 +1321,92 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_raconter_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le sac de pain craque encore un peu.
-narrateur|Une miette tombe sur la nappe à carreaux.
-narrateur|Ça sent le four du village.
-narrateur|La rue est calme, tout près.
-narrateur|Un vélo passe au loin, tout léger.
+          <t>narrateur|Une odeur de croûte traverse la rue.
+narrateur|Le four du village respire, chaud.
+narrateur|Un vélo passe au loin.
+narrateur|Ding.
+narrateur|Victorino connaît cette table.
+narrateur|La nappe à carreaux est rouge et blanche.
+narrateur|Sur la table, le sac de pain craque.
+narrateur|Le papier du sac est chaud, un peu rêche.
 narrateur|Papa coupe une tartine.
-narrateur|La croûte est dorée.
+narrateur|La croûte est dorée, un peu cassante.
+narrateur|Sur la croûte, un éclat de croûte brille.
+enfant-m|Il est doré, papa.
+papa|C'est le four, Victorino.
+maman|Tu sens le pain, toi ?
+enfant-m|Oui, maman.
+enfant-m|Je veux le dire, maintenant !
+narrateur|Papa parle à maman, près du lait.
+papa|Le vélo a sonné, dans la rue.
+maman|Oui, il était loin.
+enfant-m|Papa, le vélo !
+narrateur|Les mots de Victorino se cognent aux leurs.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose ?
+enfant-m|Le vélo, il a sonné !
+narrateur|Victorino parle trop vite.
+narrateur|Les mots tombent, mélangés.
+enfant-m|Oh.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|L'éclat de croûte tremble, puis tient.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes le pain ?
+narrateur|En ce moment, Victorino serre le sac.
+narrateur|Le papier reste chaud sous les doigts.
+maman|Tu essuies tes doigts ?
+enfant-m|Oui.
 narrateur|Maman verse un peu de lait.
-papa|Le pain est encore tiède, tu sens ?
-maman|Une petite miette a voyagé jusqu'à la nappe.
-narrateur|En ce moment, Victorino touche la croûte tiède.
-enfant-m|Elle est chaude, papa.
-papa|Une bouchée, puis on part.
-narrateur|Victorino croque.
-narrateur|La croûte fait un petit bruit.
-enfant-m|À l'école, je veux découper un rond.
-enfant-m|Un rond comme le pain.
-maman|Tu essuies tes doigts d'abord.
-narrateur|Victorino passe le torchon.
-narrateur|Le lait laisse une petite moustache blanche.
-maman|Viens.
-maman|J'essuie.
-enfant-m|Merci, maman.
-papa|Le village sent le pain, ce matin.
-maman|Tu as entendu le vélo, tout à l'heure ?
-enfant-m|Oui.
-enfant-m|Il était loin.
-papa|Tu dis bonjour à la maîtresse.
-enfant-m|Oui.
-narrateur|L'école sent le papier et le savon des mains.
-narrateur|Les chaises font un petit bruit sur le sol.
-maitresse|Bonjour.
-maitresse|On range les ciseaux, maintenant.
-enfant-m|Bonjour, maîtresse.
-narrateur|Victorino écoute.
-narrateur|Il pose les ciseaux dans le pot, les pointes en bas.
-maitresse|Merci.
-maitresse|Maintenant, on découpe un rond.
-narrateur|Victorino prend une feuille.
-narrateur|Il suit la ligne, tout doux.
-narrateur|Le rond tombe sur la table.
-enfant-m|Il ressemble au pain.
-maitresse|Oui, Victorino.
-narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, tout près de l'oreille.
+narrateur|Une moustache blanche reste sur la lèvre.
+narrateur|Une miette dore un carreau rouge.
+papa|On y va ?
+enfant-m|On y va.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Victorino.
+narrateur|Dehors, la rue sent le four.
+narrateur|Le vélo n'est plus là.
+narrateur|L'école sent le papier et le savon.
+narrateur|Les chaises font un petit bruit.
+narrateur|Victorino s'assoit près du pot.
+narrateur|Les ciseaux brillent, pointes en bas.
+narrateur|Il veut raconter le vélo.
+enfant-m|Le vélo a sonné, dans la rue !
+narrateur|Sa voix se cogne à la classe.
+narrateur|Personne ne comprend le vélo.
+narrateur|Victorino referme la bouche.
+narrateur|Un camarade s'approche.
+narrateur|Il parle près de l'oreille.
 narrateur|Victorino sent un malaise.
 narrateur|Son ventre se serre, comme un nœud.
-narrateur|Il reste assis.
-narrateur|Il pose le rond de papier près du pot.
-narrateur|Les ciseaux brillent dans le pot, tout sages.
-narrateur|Le soir, le sac de pain est encore sur la table.
+enfant-m|Je veux le dire, maintenant.
+narrateur|Il ouvre la bouche, trop vite.
+narrateur|Les mots se perdent dans la classe.
+narrateur|Personne n'entend le malaise.
+narrateur|Victorino reste assis.
+narrateur|Le nœud reste dans le ventre.
+narrateur|Le soir, le sac de pain est sur la table.
 narrateur|Ça sent le cacao et la croûte.
+narrateur|La nappe à carreaux attend.
 narrateur|La porte s'ouvre.
 maman|Te voilà.
-maman|Tu as faim ?
-narrateur|Victorino pose le rond de papier sur la nappe.
-narrateur|À côté de la miette.
-narrateur|Le ventre est encore serré.</t>
+papa|Tu as faim ?
+narrateur|Victorino pose le cartable.
+narrateur|Le ventre est serré, tout petit.
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>porte,pas</t>
+          <t>four,pain,velo</t>
         </is>
       </c>
     </row>
@@ -1418,12 +1438,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino a un malaise. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Victorino a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nino a un malaise. Que fait-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Victorino a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1433,7 +1453,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>raconter | à la maison | maman | écouter</t>
+          <t>raconter | à la maison | maman | écouter | il raconte | raconter à maman | il écoute</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1448,7 +1468,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il écoute la maîtresse. S'il a un malaise ?</t>
+          <t>Il raconte près du pain. Que fait Victorino ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1486,7 +1506,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1497,7 +1517,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1512,34 +1532,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1554,17 +1578,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_raconte_quand_les_oreilles_sont_pretes; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1597,17 +1621,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>J'ai eu un malaise, maman. Quelqu'un a parlé tout bas. On t'écoute. Assieds-toi. Victorino parle près du rond de papier. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute. Si tu as un malaise, tu viens le dire à la maison. Le nœud dans le ventre se desserre.</t>
+          <t>Victorino ouvre la bouche trop vite. Papa, un camarade, l'oreille, le nœud ! Papa n'a pas fini sa phrase. Le cacao est chaud, Victorino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Il pose les mains près du pain. Il écoute la cuisine, un instant. Le pain est là, sur la nappe. Papa pose sa tasse. Le cacao fume un peu. Maman n'a pas fini non plus. Victorino attend que le silence arrive. Sur la croûte, l'éclat de croûte brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Victorino montre son ventre. Merci, Victorino. Papa a entendu toute la phrase. Tu as faim, maintenant ? Un peu, maman. Le ventre de Victorino se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>J'ai eu un malaise, maman. Quelqu'un a parlé tout bas. On t'écoute. Assieds-toi. Victorino parle près du rond de papier. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute. Si tu as un malaise, tu viens le dire à la maison. Le nœud dans le ventre se desserre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino ouvre la bouche trop vite. Papa, un camarade, l'oreille, le nœud ! Papa n'a pas fini sa phrase. Le cacao est chaud, Victorino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Il pose les mains près du pain. Il écoute la cuisine, un instant. Le pain est là, sur la nappe. Papa pose sa tasse. Le cacao fume un peu. Maman n'a pas fini non plus. Victorino attend que le silence arrive. Sur la croûte, l'&lt;emphasis level="moderate"&gt;éclat de croûte&lt;/emphasis&gt; brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Victorino montre son ventre. Merci, Victorino. Papa a entendu toute la phrase. Tu as faim, maintenant ? Un peu, maman. Le ventre de Victorino se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nino a écouté. Il a su &lt;emphasis&gt;raconter&lt;/emphasis&gt; à la maison. Maman était là. [pause]</t>
+          <t>Victorino ouvre la bouche trop vite. Papa, un camarade, l'oreille, le nœud ! Papa n'a pas fini sa phrase. Le cacao est chaud, Victorino. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Il pose les mains près du pain. Il écoute la cuisine, un instant. Le pain est là, sur la nappe. Papa pose sa tasse. Le cacao fume un peu. Maman n'a pas fini non plus. Victorino attend que le silence arrive. Sur la croûte, l'&lt;emphasis&gt;éclat de croûte&lt;/emphasis&gt; brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé près de mon oreille. Ça a serré, ici. Victorino montre son ventre. Merci, Victorino. Papa a entendu toute la phrase. Tu as faim, maintenant ? Un peu, maman. Le ventre de Victorino se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1654,7 +1678,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1662,10 +1686,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1688,30 +1712,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>raconter</t>
+          <t>éclat de croûte</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1720,10 +1744,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1736,22 +1760,44 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_raconte_pres_du_pain; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai eu un malaise, maman.
-enfant-m|Quelqu'un a parlé tout bas.
-maman|On t'écoute.
-papa|Assieds-toi.
-narrateur|Victorino parle près du rond de papier.
-narrateur|Papa écoute.
-narrateur|Maman écoute.
-maman|Tu as bien fait de raconter.
-papa|À l'école, on écoute.
-maman|Si tu as un malaise, tu viens le dire à la maison.
-narrateur|Le nœud dans le ventre se desserre.</t>
+          <t>narrateur|Victorino ouvre la bouche trop vite.
+enfant-m|Papa, un camarade, l'oreille, le nœud !
+narrateur|Papa n'a pas fini sa phrase.
+papa|Le cacao est chaud, Victorino.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains près du pain.
+narrateur|Il écoute la cuisine, un instant.
+papa|Le pain est là, sur la nappe.
+narrateur|Papa pose sa tasse.
+maman|Le cacao fume un peu.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Victorino attend que le silence arrive.
+narrateur|Sur la croûte, l'éclat de croûte brille.
+enfant-m|Il est là.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Un camarade a parlé près de mon oreille.
+enfant-m|Ça a serré, ici.
+narrateur|Victorino montre son ventre.
+papa|Merci, Victorino.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as faim, maintenant ?
+enfant-m|Un peu, maman.
+narrateur|Le ventre de Victorino se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pain,cacao</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1824,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Tu as fini ta tartine du soir ? Oui, maman. Une miette reste sur la nappe. Victorino rit un peu. La miette a voyagé encore. Maman pose une pomme et un morceau de pain. Viens t'asseoir, Victorino. Victorino s'assoit. La chaise est stable. Tes pieds touchent la barre ? Oui, papa. Le pain craque encore, tout doux. Mon rond de papier est là. On le pose près du vrai pain. Les deux ronds se regardent. Merci, maman. Merci, papa.</t>
+          <t>Tu t'assois ? Victorino s'assoit près du pain. Une tartine ? Oui, une tartine. Papa coupe la croûte. Victorino veut tout dire d'un coup. Et le vélo, et l'école aussi ! Les mots se bousculent. Attends. Victorino s'arrête. Il prend une bouchée. La croûte craque sous les dents. Le vélo a sonné, ce matin. Tu l'as entendu, toi ? Oui, loin dans la rue. Et à l'école ? J'ai gardé le nœud. Je le dis ici. La chaleur touche les joues de Victorino. On est bien, ici ? Oui, près du pain. Victorino sent le beurre sur ses doigts. On mange ici. Oui, ici.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Tu as fini ta tartine du soir ? Oui, maman. Une miette reste sur la nappe. Victorino rit un peu. La miette a voyagé encore. Maman pose une pomme et un morceau de pain. Viens t'asseoir, Victorino. Victorino s'assoit. La chaise est stable. Tes pieds touchent la barre ? Oui, papa. Le pain craque encore, tout doux. Mon rond de papier est là. On le pose près du vrai pain. Les deux ronds se regardent. Merci, maman. Merci, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Tu t'assois ? Victorino s'assoit près du pain. Une tartine ? Oui, une tartine. Papa coupe la &lt;emphasis level="moderate"&gt;croûte&lt;/emphasis&gt;. Victorino veut tout dire d'un coup. Et le vélo, et l'école aussi ! Les mots se bousculent. Attends. Victorino s'arrête. Il prend une bouchée. La croûte craque sous les dents. Le vélo a sonné, ce matin. Tu l'as entendu, toi ? Oui, loin dans la rue. Et à l'école ? J'ai gardé le nœud. Je le dis ici. La chaleur touche les joues de Victorino. On est bien, ici ? Oui, près du pain. Victorino sent le beurre sur ses doigts. On mange ici. Oui, ici.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman prépare le goûter. Nino s'assoit. [pause]</t>
+          <t>Tu t'assois ? Victorino s'assoit près du pain. Une tartine ? Oui, une tartine. Papa coupe la &lt;emphasis&gt;croûte&lt;/emphasis&gt;. Victorino veut tout dire d'un coup. Et le vélo, et l'école aussi ! Les mots se bousculent. Attends. Victorino s'arrête. Il prend une bouchée. La croûte craque sous les dents. Le vélo a sonné, ce matin. Tu l'as entendu, toi ? Oui, loin dans la rue. Et à l'école ? J'ai gardé le nœud. Je le dis ici. La chaleur touche les joues de Victorino. On est bien, ici ? Oui, près du pain. Victorino sent le beurre sur ses doigts. On mange ici. Oui, ici. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,7 +1881,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1843,10 +1889,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1913,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>croûte</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1947,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1911,26 +1961,42 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=refermer_le_désir; emotion=fierté_calme et chaleur; intensite=2; destinataire=enfant; sous_texte=il_dit_une_chose_pres_du_pain; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|Tu as fini ta tartine du soir ?
-enfant-m|Oui, maman.
-narrateur|Une miette reste sur la nappe.
-narrateur|Victorino rit un peu.
-papa|La miette a voyagé encore.
-narrateur|Maman pose une pomme et un morceau de pain.
-maman|Viens t'asseoir, Victorino.
-narrateur|Victorino s'assoit.
-narrateur|La chaise est stable.
-papa|Tes pieds touchent la barre ?
-enfant-m|Oui, papa.
-narrateur|Le pain craque encore, tout doux.
-enfant-m|Mon rond de papier est là.
-maman|On le pose près du vrai pain.
-narrateur|Les deux ronds se regardent.
-enfant-m|Merci, maman.
-enfant-m|Merci, papa.</t>
+          <t>papa|Tu t'assois ?
+narrateur|Victorino s'assoit près du pain.
+maman|Une tartine ?
+enfant-m|Oui, une tartine.
+narrateur|Papa coupe la croûte.
+narrateur|Victorino veut tout dire d'un coup.
+enfant-m|Et le vélo, et l'école aussi !
+narrateur|Les mots se bousculent.
+enfant-m|Attends.
+narrateur|Victorino s'arrête.
+narrateur|Il prend une bouchée.
+narrateur|La croûte craque sous les dents.
+enfant-m|Le vélo a sonné, ce matin.
+papa|Tu l'as entendu, toi ?
+enfant-m|Oui, loin dans la rue.
+maman|Et à l'école ?
+enfant-m|J'ai gardé le nœud.
+enfant-m|Je le dis ici.
+narrateur|La chaleur touche les joues de Victorino.
+papa|On est bien, ici ?
+enfant-m|Oui, près du pain.
+narrateur|Victorino sent le beurre sur ses doigts.
+maman|On mange ici.
+enfant-m|Oui, ici.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pain,beurre</t>
         </is>
       </c>
     </row>
@@ -1957,17 +2023,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac de pain se tait. Le rond de papier reste sur la nappe. On t'a écouté, Victorino. Le pain était tiède.</t>
+          <t>Le pain était chaud. Tu es venu le dire. Tu le vois, toi ? Oui, sur la croûte. Le sac de pain se tait. Victorino sent la croûte sur sa langue. Sur la croûte, l'éclat de croûte garde une trace.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sac de pain se tait. Le rond de papier reste sur la nappe. On t'a écouté, Victorino. Le pain était tiède.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le pain était chaud. Tu es venu le dire. Tu le vois, toi ? Oui, sur la croûte. Le sac de pain se tait. Victorino sent la croûte sur sa langue. Sur la croûte, l'&lt;emphasis level="moderate"&gt;éclat de croûte&lt;/emphasis&gt; garde une trace.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le pain était chaud. Tu es venu le dire. Tu le vois, toi ? Oui, sur la croûte. Le sac de pain se tait. Victorino sent la croûte sur sa langue. Sur la croûte, l'&lt;emphasis&gt;éclat de croûte&lt;/emphasis&gt; garde une trace.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2014,7 +2080,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2022,10 +2088,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2034,12 +2100,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2048,17 +2114,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de croûte</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2067,11 +2137,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2080,27 +2150,39 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_croute_garde_une_trace; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac de pain se tait.
-narrateur|Le rond de papier reste sur la nappe.
-papa|On t'a écouté, Victorino.
-maman|Le pain était tiède.</t>
+          <t>enfant-m|Le pain était chaud.
+maman|Tu es venu le dire.
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur la croûte.
+narrateur|Le sac de pain se tait.
+narrateur|Victorino sent la croûte sur sa langue.
+narrateur|Sur la croûte, l'éclat de croûte garde une trace.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>pain</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2213,6 +2295,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>